<commit_message>
add more column in export + add more verification for customer approval date validation
</commit_message>
<xml_diff>
--- a/core/src/main/resources/excel-templates/standard-generation-excel-file-template.xlsx
+++ b/core/src/main/resources/excel-templates/standard-generation-excel-file-template.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muss/dev/cost-seiko-core/core/src/main/resources/excel-templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muss/dev/npi-seiko-core/core/src/main/resources/excel-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F4F255-E7A4-344E-B3E0-4C43FC531EE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F28BC9-D10B-1F49-8B9F-A11BAAED06FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="749" xr2:uid="{C9F70631-86D4-460D-A672-BF4D1106FF45}"/>
+    <workbookView xWindow="4280" yWindow="660" windowWidth="25960" windowHeight="18980" tabRatio="749" xr2:uid="{C9F70631-86D4-460D-A672-BF4D1106FF45}"/>
   </bookViews>
   <sheets>
-    <sheet name="Fabrication" sheetId="19" r:id="rId1"/>
+    <sheet name="Npi orders" sheetId="19" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -22,10 +22,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -100,13 +96,13 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -615,21 +611,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010049099315E98CCB42BF73A6B81E487C10" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="df55fe4f37d050e510ccee2c1adbdef1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d2592f0d-2e69-4d88-9eda-f93a1e02d3f1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29797a14f8dea13fdf553f1f03cdce76" ns2:_="">
     <xsd:import namespace="d2592f0d-2e69-4d88-9eda-f93a1e02d3f1"/>
@@ -773,24 +754,22 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9174E288-DE7D-4B2D-89C1-47E547D8A97F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841F5774-E854-4835-BDF9-7FB18D6E9DB6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{291DBB97-D44F-4070-B808-AB9096087FA8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -806,4 +785,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841F5774-E854-4835-BDF9-7FB18D6E9DB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9174E288-DE7D-4B2D-89C1-47E547D8A97F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>